<commit_message>
Agrege el envio de correos electronicos
</commit_message>
<xml_diff>
--- a/Libro1.xlsx
+++ b/Libro1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maner\OneDrive\Escritorio\sem3\lenguajes\proyecto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\PycharmProjects\Lenguajes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F624D5AB-F722-4D87-AA22-93639DE7EA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F74446E2-CA9F-4A07-B20E-4A00950C56D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D3B63391-DFFB-4905-83B3-D104C39CB9B8}"/>
+    <workbookView xWindow="1100" yWindow="1100" windowWidth="19200" windowHeight="11710" xr2:uid="{D3B63391-DFFB-4905-83B3-D104C39CB9B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,30 +20,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
-  <si>
-    <t>Cta.</t>
-  </si>
-  <si>
-    <t>Nombre Copleto</t>
-  </si>
-  <si>
-    <t>ASISTE</t>
-  </si>
-  <si>
-    <t>PIOE-B1</t>
-  </si>
-  <si>
-    <t>PIOE-B2</t>
-  </si>
-  <si>
-    <t>REGISTRO BECAS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>515149</t>
   </si>
@@ -232,13 +225,127 @@
   </si>
   <si>
     <t>ZUÑIGA FALCON  HECTOR ANDRES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clave </t>
+  </si>
+  <si>
+    <t>Num_Cuenta</t>
+  </si>
+  <si>
+    <t>Correo</t>
+  </si>
+  <si>
+    <t>nombre_completo</t>
+  </si>
+  <si>
+    <t>GOMEZ PEREZ ANGEL GABREIL</t>
+  </si>
+  <si>
+    <t>alvarezcruzlennydanahe@gmailcom</t>
+  </si>
+  <si>
+    <t>angelesperezrogeliosebastian@gmailcom</t>
+  </si>
+  <si>
+    <t>antoniolorenzosharonjimena@gmailcom</t>
+  </si>
+  <si>
+    <t>cruzcruzsebastian@gmailcom</t>
+  </si>
+  <si>
+    <t>duranchavezcamilazandily@gmailcom</t>
+  </si>
+  <si>
+    <t>escobaralvaradodulceabigail@gmailcom</t>
+  </si>
+  <si>
+    <t>estradaramirezcynthiazoe@gmailcom</t>
+  </si>
+  <si>
+    <t>florescoronamariajose@gmailcom</t>
+  </si>
+  <si>
+    <t>godinezhernandezjuanpablo@gmailcom</t>
+  </si>
+  <si>
+    <t>gonzalezbarrerakarlaalexa@gmailcom</t>
+  </si>
+  <si>
+    <t>gonzalezsanchezkimberly@gmailcom</t>
+  </si>
+  <si>
+    <t>guerreroriosbrayanalexander@gmailcom</t>
+  </si>
+  <si>
+    <t>gutierrezolverailse@gmailcom</t>
+  </si>
+  <si>
+    <t>hernandezcabreramiguelangel@gmailcom</t>
+  </si>
+  <si>
+    <t>herrejonalvarezdanielanofrith@gmailcom</t>
+  </si>
+  <si>
+    <t>juarezgarciayoanaaracely@gmailcom</t>
+  </si>
+  <si>
+    <t>lopezaguilarvalerializeth@gmailcom</t>
+  </si>
+  <si>
+    <t>lopezdejesusangeljared@gmailcom</t>
+  </si>
+  <si>
+    <t>medinamarmolejodiego@gmailcom</t>
+  </si>
+  <si>
+    <t>mezamelchordavid@gmailcom</t>
+  </si>
+  <si>
+    <t>neriaperezmichelleabigail@gmailcom</t>
+  </si>
+  <si>
+    <t>olguingarciastevengilberto@gmailcom</t>
+  </si>
+  <si>
+    <t>ramirezsanchezahmed@gmailcom</t>
+  </si>
+  <si>
+    <t>ramireztellezlizzethvalentina@gmailcom</t>
+  </si>
+  <si>
+    <t>resendizramirezfernanda@gmailcom</t>
+  </si>
+  <si>
+    <t>riveraramirezjesuseduardo@gmailcom</t>
+  </si>
+  <si>
+    <t>rodriguezjimenezdaniela@gmailcom</t>
+  </si>
+  <si>
+    <t>tobonsalasfernandaalejandra@gmailcom</t>
+  </si>
+  <si>
+    <t>torresgressluisjonathan@gmailcom</t>
+  </si>
+  <si>
+    <t>vargashernandezromina@gmailcom</t>
+  </si>
+  <si>
+    <t>villanuevacortezazulselina@gmailcom</t>
+  </si>
+  <si>
+    <t>zuñigafalconhectorandres@gmailcom</t>
+  </si>
+  <si>
+    <t>go525573@uaeh.edu.mx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +377,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -280,12 +395,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -308,35 +423,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -353,9 +486,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -393,7 +526,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -499,7 +632,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -641,7 +774,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -649,414 +782,566 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB502872-E649-4E31-9913-39A8E2CC0C3A}">
-  <dimension ref="A1:F33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="36.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="4"/>
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1234</v>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="C3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="1">
+        <v>56789</v>
+      </c>
+      <c r="E3" s="8"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="C4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5432</v>
+      </c>
+      <c r="E4" s="8"/>
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="C5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2343</v>
+      </c>
+      <c r="E5" s="8"/>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="8"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3234</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="9"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="C7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3453</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="9"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="C8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3451</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="8"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="C9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="1">
+        <v>9647</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="9"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="C10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="1">
+        <v>4267</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="9"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="C11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1345</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="8"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="C12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1243</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="C13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2223</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="9"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="C14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="1">
+        <v>9678</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B15" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="C15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="1">
+        <v>5678</v>
+      </c>
+      <c r="E15" s="8"/>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B16" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="C16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="1">
+        <v>6789</v>
+      </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B17" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="9"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="C17" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="1">
+        <v>6788</v>
+      </c>
+      <c r="E17" s="8"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>518392</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C18" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="1">
+        <v>6789</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="9"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="1">
+        <v>7899</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="9"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1330</v>
+      </c>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="8"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="6">
-        <v>518392</v>
-      </c>
-      <c r="B18" s="6" t="s">
+      <c r="B21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="9"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="C21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="1">
+        <v>1111</v>
+      </c>
+      <c r="E21" s="8"/>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B22" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="9"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="C22" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="1">
+        <v>2222</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B23" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="9"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="C23" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" s="1">
+        <v>3333</v>
+      </c>
+      <c r="E23" s="8"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="8"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="C24" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="1">
+        <v>4444</v>
+      </c>
+      <c r="E24" s="8"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="9"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="C25" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D25" s="1">
+        <v>5555</v>
+      </c>
+      <c r="E25" s="8"/>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B26" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="8"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="C26" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="D26" s="1">
+        <v>6666</v>
+      </c>
+      <c r="E26" s="8"/>
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B27" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="8"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+      <c r="C27" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="1">
+        <v>7777</v>
+      </c>
+      <c r="E27" s="8"/>
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="8"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="C28" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="D28" s="1">
+        <v>8888</v>
+      </c>
+      <c r="E28" s="8"/>
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B29" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="9"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="C29" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="1">
+        <v>9999</v>
+      </c>
+      <c r="E29" s="8"/>
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B30" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="1"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="9"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+      <c r="C30" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="1">
+        <v>1212</v>
+      </c>
+      <c r="E30" s="8"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B31" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="9"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+      <c r="C31" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" s="1">
+        <v>2323</v>
+      </c>
+      <c r="E31" s="8"/>
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B32" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="1"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="8"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="C32" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32" s="1">
+        <v>4355</v>
+      </c>
+      <c r="E32" s="8"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B33" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="8"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="1"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="9"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C32" s="1"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="8"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="C33" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D33" s="1">
+        <v>5666</v>
+      </c>
+      <c r="E33" s="8"/>
+      <c r="F33" s="7"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>525573</v>
+      </c>
+      <c r="B34" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C33" s="1"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="9"/>
+      <c r="C34" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="12">
+        <v>1234</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C34" r:id="rId1" xr:uid="{F25BC93C-9548-4B54-AB8D-6824A43AF11E}"/>
+    <hyperlink ref="C33" r:id="rId2" xr:uid="{B7AD3325-EFD0-4291-8861-E7B8CCAF9A07}"/>
+    <hyperlink ref="C31" r:id="rId3" xr:uid="{890D6668-DF09-4C8E-9792-F4A19AD3F8E7}"/>
+    <hyperlink ref="C32" r:id="rId4" xr:uid="{C6076C3C-0F17-4868-9470-1BB483D05E17}"/>
+    <hyperlink ref="C29" r:id="rId5" xr:uid="{ADEC5C2E-D526-4415-902E-D727A35AEBC9}"/>
+    <hyperlink ref="C30" r:id="rId6" xr:uid="{467D8063-4589-4246-BCFD-85AB53BA9670}"/>
+    <hyperlink ref="C28" r:id="rId7" xr:uid="{A3A7D0A8-67F6-405E-9F16-6F255E1E47A3}"/>
+    <hyperlink ref="C27" r:id="rId8" xr:uid="{E6DCF147-B36A-4983-B250-B19636A70418}"/>
+    <hyperlink ref="C25" r:id="rId9" xr:uid="{98AA9398-EF05-4B17-B08A-F217CE20F611}"/>
+    <hyperlink ref="C26" r:id="rId10" xr:uid="{FCEB0F08-37BA-464A-BE9B-A7F663F79FDA}"/>
+    <hyperlink ref="C24" r:id="rId11" xr:uid="{5816473A-C870-4051-8BFF-68B5CC3CB9CD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
reparando pendejadas de david
</commit_message>
<xml_diff>
--- a/Libro1.xlsx
+++ b/Libro1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\PycharmProjects\Lenguajes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F74446E2-CA9F-4A07-B20E-4A00950C56D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3BB795-1023-48E0-8C14-4C2FD175010C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="1100" windowWidth="19200" windowHeight="11710" xr2:uid="{D3B63391-DFFB-4905-83B3-D104C39CB9B8}"/>
   </bookViews>
@@ -338,14 +338,14 @@
     <t>zuñigafalconhectorandres@gmailcom</t>
   </si>
   <si>
-    <t>go525573@uaeh.edu.mx</t>
+    <t>angelgabrielgomezperez72@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,6 +381,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -439,7 +447,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -467,6 +475,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -782,7 +791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB502872-E649-4E31-9913-39A8E2CC0C3A}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="36.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1326,6 +1335,9 @@
       <c r="D34" s="12">
         <v>1234</v>
       </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B35" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>